<commit_message>
Refactor education management components to include training codes and improve label formatting
- Updated TopEgitimlerChart to use "etiket" instead of "egitimAdi" for better data representation.
- Enhanced EgitimPlani components to utilize formatEgitimLabel for consistent training name formatting.
- Modified PlanEkleModal to display training codes alongside names.
- Improved Raporlar component to handle training codes in reports and display formatted labels.
- Updated TalepDetay and TalepForm components to include training codes in their displays.
- Added functionality to manage training categories in useEgitimData, allowing for dynamic category updates.
- Enhanced helper functions to format training labels and signatures, ensuring consistent presentation across the application.
- Adjusted CSS styles for better layout and spacing in various components.
</commit_message>
<xml_diff>
--- a/egitim-plani/public/ornek-talep-aktarim.xlsx
+++ b/egitim-plani/public/ornek-talep-aktarim.xlsx
@@ -397,110 +397,188 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:S3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Y?netici Ad?</v>
+        <v>YoneticiAdi</v>
       </c>
       <c r="B1" t="str">
-        <v>Y?netici E-posta</v>
+        <v>YoneticiEposta</v>
       </c>
       <c r="C1" t="str">
         <v>GMY</v>
       </c>
       <c r="D1" t="str">
-        <v>?al??an Ad?</v>
+        <v>CalisanAdi</v>
       </c>
       <c r="E1" t="str">
-        <v>?al??an Sicil No</v>
+        <v>CalisanKullaniciKodu</v>
       </c>
       <c r="F1" t="str">
-        <v>?al??an Kullan?c? Kodu</v>
+        <v>CalisanSicilNo</v>
       </c>
       <c r="G1" t="str">
+        <v>Egitim1Kodu</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Egitim1Adi</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Egitim1Kategori</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Egitim2Kodu</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Egitim2Adi</v>
+      </c>
+      <c r="L1" t="str">
+        <v>Egitim2Kategori</v>
+      </c>
+      <c r="M1" t="str">
+        <v>Egitim3Kodu</v>
+      </c>
+      <c r="N1" t="str">
+        <v>Egitim3Adi</v>
+      </c>
+      <c r="O1" t="str">
+        <v>Egitim3Kategori</v>
+      </c>
+      <c r="P1" t="str">
+        <v>Egitim4Kodu</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>Egitim4Adi</v>
+      </c>
+      <c r="R1" t="str">
+        <v>Egitim4Kategori</v>
+      </c>
+      <c r="S1" t="str">
         <v>Notlar</v>
-      </c>
-      <c r="H1" t="str">
-        <v>E?itim 1 Ad?</v>
-      </c>
-      <c r="I1" t="str">
-        <v>E?itim 1 Kategori</v>
-      </c>
-      <c r="J1" t="str">
-        <v>E?itim 2 Ad?</v>
-      </c>
-      <c r="K1" t="str">
-        <v>E?itim 2 Kategori</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Ay?e Y?lmaz</v>
+        <v>Ayse Yilmaz</v>
       </c>
       <c r="B2" t="str">
-        <v>ayse.yilmaz@sirket.com</v>
+        <v>ayse.yilmaz@ornek.com</v>
       </c>
       <c r="C2" t="str">
         <v>Teknoloji GMY</v>
       </c>
       <c r="D2" t="str">
-        <v>Mehmet Demir</v>
+        <v>Mert Kaya</v>
       </c>
       <c r="E2" t="str">
-        <v>45821</v>
+        <v>mkaya</v>
       </c>
       <c r="F2" t="str">
-        <v>m.demir</v>
+        <v>100245</v>
       </c>
       <c r="G2" t="str">
-        <v>Backend ekibi i?in ?ncelikli ihtiya?.</v>
+        <v>TE_001</v>
       </c>
       <c r="H2" t="str">
-        <v>React ?leri Seviye</v>
+        <v>Temel Network</v>
       </c>
       <c r="I2" t="str">
         <v>Teknik</v>
       </c>
       <c r="J2" t="str">
-        <v>Etkili Sunum Teknikleri</v>
+        <v>TE_014</v>
       </c>
       <c r="K2" t="str">
-        <v>Ki?isel Geli?im</v>
+        <v>Windows Server Temelleri</v>
+      </c>
+      <c r="L2" t="str">
+        <v>Teknik</v>
+      </c>
+      <c r="M2" t="str">
+        <v/>
+      </c>
+      <c r="N2" t="str">
+        <v/>
+      </c>
+      <c r="O2" t="str">
+        <v/>
+      </c>
+      <c r="P2" t="str">
+        <v/>
+      </c>
+      <c r="Q2" t="str">
+        <v/>
+      </c>
+      <c r="R2" t="str">
+        <v/>
+      </c>
+      <c r="S2" t="str">
+        <v>Yil icinde oncelikli teknik gelisim talebi</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Selin Kaya</v>
+        <v>Burak Demir</v>
       </c>
       <c r="B3" t="str">
-        <v>selin.kaya@sirket.com</v>
+        <v>burak.demir@ornek.com</v>
       </c>
       <c r="C3" t="str">
-        <v>Sat?? GMY</v>
+        <v>Satis GMY</v>
       </c>
       <c r="D3" t="str">
-        <v>Zeynep Acar</v>
+        <v>Ece Arslan</v>
       </c>
       <c r="E3" t="str">
-        <v>52710</v>
+        <v>earslan</v>
       </c>
       <c r="F3" t="str">
-        <v>z.acar</v>
+        <v>100318</v>
       </c>
       <c r="G3" t="str">
-        <v>Yeni m??teri kazan?m? odakl? e?itim talebi.</v>
+        <v>SP_003</v>
       </c>
       <c r="H3" t="str">
-        <v>?leri M?zakere Teknikleri</v>
+        <v>Ileri Satis Teknikleri</v>
       </c>
       <c r="I3" t="str">
-        <v>Sat?? &amp; Pazarlama</v>
+        <v>Satis &amp; Pazarlama</v>
+      </c>
+      <c r="J3" t="str">
+        <v>LD_002</v>
+      </c>
+      <c r="K3" t="str">
+        <v>Sunum ve Etki Becerileri</v>
+      </c>
+      <c r="L3" t="str">
+        <v>Kisisel Gelisim</v>
+      </c>
+      <c r="M3" t="str">
+        <v/>
+      </c>
+      <c r="N3" t="str">
+        <v/>
+      </c>
+      <c r="O3" t="str">
+        <v/>
+      </c>
+      <c r="P3" t="str">
+        <v/>
+      </c>
+      <c r="Q3" t="str">
+        <v/>
+      </c>
+      <c r="R3" t="str">
+        <v/>
+      </c>
+      <c r="S3" t="str">
+        <v>Bolgesel satis ekibi icin gelisim talebi</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: enhance admin panel with catalog search and filtering; update constants and improve styling
</commit_message>
<xml_diff>
--- a/egitim-plani/public/ornek-talep-aktarim.xlsx
+++ b/egitim-plani/public/ornek-talep-aktarim.xlsx
@@ -3,7 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Talepler" sheetId="1" r:id="rId1"/>
+    <sheet name="Ornek Talepler" sheetId="1" r:id="rId1"/>
+    <sheet name="Referans Listeler" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
 </file>
@@ -397,7 +398,28 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S3"/>
+  <dimension ref="A1:S8"/>
+  <cols>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="22.83203125" customWidth="1"/>
+    <col min="3" max="3" width="22.83203125" customWidth="1"/>
+    <col min="4" max="4" width="22.83203125" customWidth="1"/>
+    <col min="5" max="5" width="22.83203125" customWidth="1"/>
+    <col min="6" max="6" width="22.83203125" customWidth="1"/>
+    <col min="7" max="7" width="22.83203125" customWidth="1"/>
+    <col min="8" max="8" width="22.83203125" customWidth="1"/>
+    <col min="9" max="9" width="22.83203125" customWidth="1"/>
+    <col min="10" max="10" width="22.83203125" customWidth="1"/>
+    <col min="11" max="11" width="22.83203125" customWidth="1"/>
+    <col min="12" max="12" width="22.83203125" customWidth="1"/>
+    <col min="13" max="13" width="22.83203125" customWidth="1"/>
+    <col min="14" max="14" width="22.83203125" customWidth="1"/>
+    <col min="15" max="15" width="22.83203125" customWidth="1"/>
+    <col min="16" max="16" width="22.83203125" customWidth="1"/>
+    <col min="17" max="17" width="22.83203125" customWidth="1"/>
+    <col min="18" max="18" width="22.83203125" customWidth="1"/>
+    <col min="19" max="19" width="22.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -463,58 +485,58 @@
         <v>Ayse Yilmaz</v>
       </c>
       <c r="B2" t="str">
-        <v>ayse.yilmaz@ornek.com</v>
+        <v>ayse.yilmaz@firma.com</v>
       </c>
       <c r="C2" t="str">
-        <v>Teknoloji GMY</v>
+        <v>Mali Yönetim Direktörlüğü</v>
       </c>
       <c r="D2" t="str">
-        <v>Mert Kaya</v>
+        <v>Mert Acar</v>
       </c>
       <c r="E2" t="str">
-        <v>mkaya</v>
+        <v>mert.acar</v>
       </c>
       <c r="F2" t="str">
-        <v>100245</v>
+        <v>1001</v>
       </c>
       <c r="G2" t="str">
-        <v>TE_001</v>
+        <v>TEKEGI_001</v>
       </c>
       <c r="H2" t="str">
-        <v>Temel Network</v>
+        <v>Teknik Eğitimler Temel Programi</v>
       </c>
       <c r="I2" t="str">
-        <v>Teknik</v>
+        <v>Teknik Eğitimler</v>
       </c>
       <c r="J2" t="str">
-        <v>TE_014</v>
+        <v>KISGEL_003</v>
       </c>
       <c r="K2" t="str">
-        <v>Windows Server Temelleri</v>
+        <v>Kişisel Gelişim Eğitimleri Temel Programi</v>
       </c>
       <c r="L2" t="str">
-        <v>Teknik</v>
+        <v>Kişisel Gelişim Eğitimleri</v>
       </c>
       <c r="M2" t="str">
-        <v/>
+        <v>MESGEL_006</v>
       </c>
       <c r="N2" t="str">
-        <v/>
+        <v>Mesleki Gelişim Eğitimleri Uygulama Atolyesi</v>
       </c>
       <c r="O2" t="str">
-        <v/>
+        <v>Mesleki Gelişim Eğitimleri</v>
       </c>
       <c r="P2" t="str">
-        <v/>
+        <v>SER_008</v>
       </c>
       <c r="Q2" t="str">
-        <v/>
+        <v>Sertifika Uygulama Atolyesi</v>
       </c>
       <c r="R2" t="str">
-        <v/>
+        <v>Sertifika</v>
       </c>
       <c r="S2" t="str">
-        <v>Yil icinde oncelikli teknik gelisim talebi</v>
+        <v>Mali Yönetim Direktörlüğü icin guncel ornek talep satiri. Tum kategori listesinden egitimler dagitildi.</v>
       </c>
     </row>
     <row r="3">
@@ -522,63 +544,682 @@
         <v>Burak Demir</v>
       </c>
       <c r="B3" t="str">
-        <v>burak.demir@ornek.com</v>
+        <v>burak.demir@firma.com</v>
       </c>
       <c r="C3" t="str">
-        <v>Satis GMY</v>
+        <v>İnsan Kaynakları Direktörlüğü</v>
       </c>
       <c r="D3" t="str">
-        <v>Ece Arslan</v>
+        <v>Zeynep Kaya</v>
       </c>
       <c r="E3" t="str">
-        <v>earslan</v>
+        <v>zeynep.kaya</v>
       </c>
       <c r="F3" t="str">
-        <v>100318</v>
+        <v>1002</v>
       </c>
       <c r="G3" t="str">
-        <v>SP_003</v>
+        <v>KISGEL_003</v>
       </c>
       <c r="H3" t="str">
-        <v>Ileri Satis Teknikleri</v>
+        <v>Kişisel Gelişim Eğitimleri Temel Programi</v>
       </c>
       <c r="I3" t="str">
-        <v>Satis &amp; Pazarlama</v>
+        <v>Kişisel Gelişim Eğitimleri</v>
       </c>
       <c r="J3" t="str">
-        <v>LD_002</v>
+        <v>MESGEL_005</v>
       </c>
       <c r="K3" t="str">
-        <v>Sunum ve Etki Becerileri</v>
+        <v>Mesleki Gelişim Eğitimleri Temel Programi</v>
       </c>
       <c r="L3" t="str">
-        <v>Kisisel Gelisim</v>
+        <v>Mesleki Gelişim Eğitimleri</v>
       </c>
       <c r="M3" t="str">
-        <v/>
+        <v>SER_008</v>
       </c>
       <c r="N3" t="str">
-        <v/>
+        <v>Sertifika Uygulama Atolyesi</v>
       </c>
       <c r="O3" t="str">
-        <v/>
+        <v>Sertifika</v>
       </c>
       <c r="P3" t="str">
-        <v/>
+        <v>KON_010</v>
       </c>
       <c r="Q3" t="str">
-        <v/>
+        <v>Konferans Uygulama Atolyesi</v>
       </c>
       <c r="R3" t="str">
-        <v/>
+        <v>Konferans</v>
       </c>
       <c r="S3" t="str">
-        <v>Bolgesel satis ekibi icin gelisim talebi</v>
+        <v>İnsan Kaynakları Direktörlüğü icin guncel ornek talep satiri. Tum kategori listesinden egitimler dagitildi.</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Selin Arslan</v>
+      </c>
+      <c r="B4" t="str">
+        <v>selin.arslan@firma.com</v>
+      </c>
+      <c r="C4" t="str">
+        <v>KKST GMY</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Onur Can</v>
+      </c>
+      <c r="E4" t="str">
+        <v>onur.can</v>
+      </c>
+      <c r="F4" t="str">
+        <v>1003</v>
+      </c>
+      <c r="G4" t="str">
+        <v>MESGEL_005</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Mesleki Gelişim Eğitimleri Temel Programi</v>
+      </c>
+      <c r="I4" t="str">
+        <v>Mesleki Gelişim Eğitimleri</v>
+      </c>
+      <c r="J4" t="str">
+        <v>SER_007</v>
+      </c>
+      <c r="K4" t="str">
+        <v>Sertifika Temel Programi</v>
+      </c>
+      <c r="L4" t="str">
+        <v>Sertifika</v>
+      </c>
+      <c r="M4" t="str">
+        <v>KON_010</v>
+      </c>
+      <c r="N4" t="str">
+        <v>Konferans Uygulama Atolyesi</v>
+      </c>
+      <c r="O4" t="str">
+        <v>Konferans</v>
+      </c>
+      <c r="P4" t="str">
+        <v>TEKEGI_002</v>
+      </c>
+      <c r="Q4" t="str">
+        <v>Teknik Eğitimler Uygulama Atolyesi</v>
+      </c>
+      <c r="R4" t="str">
+        <v>Teknik Eğitimler</v>
+      </c>
+      <c r="S4" t="str">
+        <v>KKST GMY icin guncel ornek talep satiri. Tum kategori listesinden egitimler dagitildi.</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Deniz Sahin</v>
+      </c>
+      <c r="B5" t="str">
+        <v>deniz.sahin@firma.com</v>
+      </c>
+      <c r="C5" t="str">
+        <v>SOPT GMY</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Elif Candan</v>
+      </c>
+      <c r="E5" t="str">
+        <v>elif.candan</v>
+      </c>
+      <c r="F5" t="str">
+        <v>1004</v>
+      </c>
+      <c r="G5" t="str">
+        <v>SER_007</v>
+      </c>
+      <c r="H5" t="str">
+        <v>Sertifika Temel Programi</v>
+      </c>
+      <c r="I5" t="str">
+        <v>Sertifika</v>
+      </c>
+      <c r="J5" t="str">
+        <v>KON_009</v>
+      </c>
+      <c r="K5" t="str">
+        <v>Konferans Temel Programi</v>
+      </c>
+      <c r="L5" t="str">
+        <v>Konferans</v>
+      </c>
+      <c r="M5" t="str">
+        <v>TEKEGI_002</v>
+      </c>
+      <c r="N5" t="str">
+        <v>Teknik Eğitimler Uygulama Atolyesi</v>
+      </c>
+      <c r="O5" t="str">
+        <v>Teknik Eğitimler</v>
+      </c>
+      <c r="P5" t="str">
+        <v>KISGEL_004</v>
+      </c>
+      <c r="Q5" t="str">
+        <v>Kişisel Gelişim Eğitimleri Uygulama Atolyesi</v>
+      </c>
+      <c r="R5" t="str">
+        <v>Kişisel Gelişim Eğitimleri</v>
+      </c>
+      <c r="S5" t="str">
+        <v>SOPT GMY icin guncel ornek talep satiri. Tum kategori listesinden egitimler dagitildi.</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Gizem Kurt</v>
+      </c>
+      <c r="B6" t="str">
+        <v>gizem.kurt@firma.com</v>
+      </c>
+      <c r="C6" t="str">
+        <v>BİT GMY</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Can Eren</v>
+      </c>
+      <c r="E6" t="str">
+        <v>can.eren</v>
+      </c>
+      <c r="F6" t="str">
+        <v>1005</v>
+      </c>
+      <c r="G6" t="str">
+        <v>KON_009</v>
+      </c>
+      <c r="H6" t="str">
+        <v>Konferans Temel Programi</v>
+      </c>
+      <c r="I6" t="str">
+        <v>Konferans</v>
+      </c>
+      <c r="J6" t="str">
+        <v>TEKEGI_001</v>
+      </c>
+      <c r="K6" t="str">
+        <v>Teknik Eğitimler Temel Programi</v>
+      </c>
+      <c r="L6" t="str">
+        <v>Teknik Eğitimler</v>
+      </c>
+      <c r="M6" t="str">
+        <v>KISGEL_004</v>
+      </c>
+      <c r="N6" t="str">
+        <v>Kişisel Gelişim Eğitimleri Uygulama Atolyesi</v>
+      </c>
+      <c r="O6" t="str">
+        <v>Kişisel Gelişim Eğitimleri</v>
+      </c>
+      <c r="P6" t="str">
+        <v>MESGEL_006</v>
+      </c>
+      <c r="Q6" t="str">
+        <v>Mesleki Gelişim Eğitimleri Uygulama Atolyesi</v>
+      </c>
+      <c r="R6" t="str">
+        <v>Mesleki Gelişim Eğitimleri</v>
+      </c>
+      <c r="S6" t="str">
+        <v>BİT GMY icin guncel ornek talep satiri. Tum kategori listesinden egitimler dagitildi.</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Emre Tekin</v>
+      </c>
+      <c r="B7" t="str">
+        <v>emre.tekin@firma.com</v>
+      </c>
+      <c r="C7" t="str">
+        <v>KG GMY</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Derya Ozturk</v>
+      </c>
+      <c r="E7" t="str">
+        <v>derya.ozturk</v>
+      </c>
+      <c r="F7" t="str">
+        <v>1006</v>
+      </c>
+      <c r="G7" t="str">
+        <v>TEKEGI_001</v>
+      </c>
+      <c r="H7" t="str">
+        <v>Teknik Eğitimler Temel Programi</v>
+      </c>
+      <c r="I7" t="str">
+        <v>Teknik Eğitimler</v>
+      </c>
+      <c r="J7" t="str">
+        <v>KISGEL_003</v>
+      </c>
+      <c r="K7" t="str">
+        <v>Kişisel Gelişim Eğitimleri Temel Programi</v>
+      </c>
+      <c r="L7" t="str">
+        <v>Kişisel Gelişim Eğitimleri</v>
+      </c>
+      <c r="M7" t="str">
+        <v>MESGEL_006</v>
+      </c>
+      <c r="N7" t="str">
+        <v>Mesleki Gelişim Eğitimleri Uygulama Atolyesi</v>
+      </c>
+      <c r="O7" t="str">
+        <v>Mesleki Gelişim Eğitimleri</v>
+      </c>
+      <c r="P7" t="str">
+        <v>SER_008</v>
+      </c>
+      <c r="Q7" t="str">
+        <v>Sertifika Uygulama Atolyesi</v>
+      </c>
+      <c r="R7" t="str">
+        <v>Sertifika</v>
+      </c>
+      <c r="S7" t="str">
+        <v>KG GMY icin guncel ornek talep satiri. Tum kategori listesinden egitimler dagitildi.</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Pelin Gunes</v>
+      </c>
+      <c r="B8" t="str">
+        <v>pelin.gunes@firma.com</v>
+      </c>
+      <c r="C8" t="str">
+        <v>UİGP GMY</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Hakan Yuce</v>
+      </c>
+      <c r="E8" t="str">
+        <v>hakan.yuce</v>
+      </c>
+      <c r="F8" t="str">
+        <v>1007</v>
+      </c>
+      <c r="G8" t="str">
+        <v>KISGEL_003</v>
+      </c>
+      <c r="H8" t="str">
+        <v>Kişisel Gelişim Eğitimleri Temel Programi</v>
+      </c>
+      <c r="I8" t="str">
+        <v>Kişisel Gelişim Eğitimleri</v>
+      </c>
+      <c r="J8" t="str">
+        <v>MESGEL_005</v>
+      </c>
+      <c r="K8" t="str">
+        <v>Mesleki Gelişim Eğitimleri Temel Programi</v>
+      </c>
+      <c r="L8" t="str">
+        <v>Mesleki Gelişim Eğitimleri</v>
+      </c>
+      <c r="M8" t="str">
+        <v>SER_008</v>
+      </c>
+      <c r="N8" t="str">
+        <v>Sertifika Uygulama Atolyesi</v>
+      </c>
+      <c r="O8" t="str">
+        <v>Sertifika</v>
+      </c>
+      <c r="P8" t="str">
+        <v>KON_010</v>
+      </c>
+      <c r="Q8" t="str">
+        <v>Konferans Uygulama Atolyesi</v>
+      </c>
+      <c r="R8" t="str">
+        <v>Konferans</v>
+      </c>
+      <c r="S8" t="str">
+        <v>UİGP GMY icin guncel ornek talep satiri. Tum kategori listesinden egitimler dagitildi.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S8"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E18"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="30.83203125" customWidth="1"/>
+    <col min="3" max="3" width="16.83203125" customWidth="1"/>
+    <col min="4" max="4" width="34.83203125" customWidth="1"/>
+    <col min="5" max="5" width="36.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Tip</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Deger</v>
+      </c>
+      <c r="C1" t="str">
+        <v>OrnekKod</v>
+      </c>
+      <c r="D1" t="str">
+        <v>OrnekEgitim</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Aciklama</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>GMY</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Mali Yönetim Direktörlüğü</v>
+      </c>
+      <c r="C2" t="str">
+        <v/>
+      </c>
+      <c r="D2" t="str">
+        <v/>
+      </c>
+      <c r="E2" t="str">
+        <v>Sistemde kayitli 1. GMY</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>GMY</v>
+      </c>
+      <c r="B3" t="str">
+        <v>İnsan Kaynakları Direktörlüğü</v>
+      </c>
+      <c r="C3" t="str">
+        <v/>
+      </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
+      <c r="E3" t="str">
+        <v>Sistemde kayitli 2. GMY</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>GMY</v>
+      </c>
+      <c r="B4" t="str">
+        <v>KKST GMY</v>
+      </c>
+      <c r="C4" t="str">
+        <v/>
+      </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
+      <c r="E4" t="str">
+        <v>Sistemde kayitli 3. GMY</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>GMY</v>
+      </c>
+      <c r="B5" t="str">
+        <v>SOPT GMY</v>
+      </c>
+      <c r="C5" t="str">
+        <v/>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+      <c r="E5" t="str">
+        <v>Sistemde kayitli 4. GMY</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>GMY</v>
+      </c>
+      <c r="B6" t="str">
+        <v>BİT GMY</v>
+      </c>
+      <c r="C6" t="str">
+        <v/>
+      </c>
+      <c r="D6" t="str">
+        <v/>
+      </c>
+      <c r="E6" t="str">
+        <v>Sistemde kayitli 5. GMY</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>GMY</v>
+      </c>
+      <c r="B7" t="str">
+        <v>KG GMY</v>
+      </c>
+      <c r="C7" t="str">
+        <v/>
+      </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
+      <c r="E7" t="str">
+        <v>Sistemde kayitli 6. GMY</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>GMY</v>
+      </c>
+      <c r="B8" t="str">
+        <v>UİGP GMY</v>
+      </c>
+      <c r="C8" t="str">
+        <v/>
+      </c>
+      <c r="D8" t="str">
+        <v/>
+      </c>
+      <c r="E8" t="str">
+        <v>Sistemde kayitli 7. GMY</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Kategori</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Teknik Eğitimler</v>
+      </c>
+      <c r="C9" t="str">
+        <v>TEKEGI_001</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Teknik Eğitimler Temel Programi</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Iceri aktarim icin birincil ornek</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Kategori</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Teknik Eğitimler</v>
+      </c>
+      <c r="C10" t="str">
+        <v>TEKEGI_002</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Teknik Eğitimler Uygulama Atolyesi</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Iceri aktarim icin ikinci ornek</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Kategori</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Kişisel Gelişim Eğitimleri</v>
+      </c>
+      <c r="C11" t="str">
+        <v>KISGEL_003</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Kişisel Gelişim Eğitimleri Temel Programi</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Iceri aktarim icin birincil ornek</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Kategori</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Kişisel Gelişim Eğitimleri</v>
+      </c>
+      <c r="C12" t="str">
+        <v>KISGEL_004</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Kişisel Gelişim Eğitimleri Uygulama Atolyesi</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Iceri aktarim icin ikinci ornek</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Kategori</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Mesleki Gelişim Eğitimleri</v>
+      </c>
+      <c r="C13" t="str">
+        <v>MESGEL_005</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Mesleki Gelişim Eğitimleri Temel Programi</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Iceri aktarim icin birincil ornek</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Kategori</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Mesleki Gelişim Eğitimleri</v>
+      </c>
+      <c r="C14" t="str">
+        <v>MESGEL_006</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Mesleki Gelişim Eğitimleri Uygulama Atolyesi</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Iceri aktarim icin ikinci ornek</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Kategori</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Sertifika</v>
+      </c>
+      <c r="C15" t="str">
+        <v>SER_007</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Sertifika Temel Programi</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Iceri aktarim icin birincil ornek</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>Kategori</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Sertifika</v>
+      </c>
+      <c r="C16" t="str">
+        <v>SER_008</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Sertifika Uygulama Atolyesi</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Iceri aktarim icin ikinci ornek</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Kategori</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Konferans</v>
+      </c>
+      <c r="C17" t="str">
+        <v>KON_009</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Konferans Temel Programi</v>
+      </c>
+      <c r="E17" t="str">
+        <v>Iceri aktarim icin birincil ornek</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Kategori</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Konferans</v>
+      </c>
+      <c r="C18" t="str">
+        <v>KON_010</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Konferans Uygulama Atolyesi</v>
+      </c>
+      <c r="E18" t="str">
+        <v>Iceri aktarim icin ikinci ornek</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E18"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>